<commit_message>
New result Fri & git ignore update
</commit_message>
<xml_diff>
--- a/Result/10-25-25/NASDAQstock_10-25-25period252RS90.xlsx
+++ b/Result/10-25-25/NASDAQstock_10-25-25period252RS90.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kelvinyue/Desktop/Coding Project/StockAnalysis/Result/10-25-25/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B449B1E-D137-8A42-AAA2-314EA3E9B547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{475EDB50-CAE5-BD49-8802-13B74D4454E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -6225,7 +6225,7 @@
       </c>
     </row>
     <row r="41" spans="1:42">
-      <c r="A41" t="s">
+      <c r="A41" s="8" t="s">
         <v>136</v>
       </c>
       <c r="B41">

</xml_diff>